<commit_message>
Split gravier into 5/15 and 5/25, add separate coffrage materiel workbook
- Commande de matériaux: gravier now split 1/3 (5/15) - 2/3 (5/25) per
  user's requested proportion, instead of one combined column.
- New workbook: commande de matériel de coffrage (planches, chevrons,
  contre-plaqué 15mm, pointes) extracted from each dalot's RECAP COFFRAGE
  sheet, in the same IST-style layout.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XXvsDUHNMYAkhaZfGs3NXn
</commit_message>
<xml_diff>
--- a/output/Commande_Materiaux_Dalots_Cafe_Cacao.xlsx
+++ b/output/Commande_Materiaux_Dalots_Cafe_Cacao.xlsx
@@ -195,11 +195,11 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -304,6 +304,7 @@
   <authors>
     <author>Note</author>
     <author>Source</author>
+    <author>Repartition</author>
   </authors>
   <commentList>
     <comment ref="D3" authorId="0" shapeId="0">
@@ -311,7 +312,7 @@
         <t>A renseigner : date d'elaboration de la commande.</t>
       </text>
     </comment>
-    <comment ref="M3" authorId="0" shapeId="0">
+    <comment ref="N3" authorId="0" shapeId="0">
       <text>
         <t>A renseigner : numero de la Demande de Sortie (DS).</t>
       </text>
@@ -321,7 +322,7 @@
         <t>A renseigner : reference / numero du marche.</t>
       </text>
     </comment>
-    <comment ref="M4" authorId="0" shapeId="0">
+    <comment ref="N4" authorId="0" shapeId="0">
       <text>
         <t>Taux de perte/chutes (mis pour information, comme dans le modele fourni). Les quantites du tableau ci-dessous sont les BESOINS NETS extraits des fiches de calcul (feuilles 'RECAP MATERIAUX' / 'MATERIAUX PRO' / 'RECAP FER' des fichiers Excel de chaque dalot), SANS majoration de perte. Appliquer ce taux manuellement si une commande majoree est necessaire.</t>
       </text>
@@ -331,14 +332,29 @@
         <t>Source : DALOT_2X2_L_7.00_ml.xlsx, feuille 'MATERIAUX PRO' (ligne TOTAL) pour Ciment/Sable/Gravier, et 'RECAP FER' colonne BOTTES pour les aciers.</t>
       </text>
     </comment>
+    <comment ref="F13" authorId="2" shapeId="0">
+      <text>
+        <t>Gravier total extrait de la source : 54.01 T, reparti ici 1/3 (5/15) - 2/3 (5/25) a la demande de l'utilisateur (le fichier source ne distingue pas les 2 granulometries).</t>
+      </text>
+    </comment>
     <comment ref="C14" authorId="1" shapeId="0">
       <text>
         <t>Source : DALOT_3X2_L7.00_ml.xlsx, feuille 'MATERIAUX PRO' (ligne TOTAL) pour Ciment/Sable/Gravier, et 'RECAP FER' colonne BOTTES pour les aciers.</t>
       </text>
     </comment>
+    <comment ref="F14" authorId="2" shapeId="0">
+      <text>
+        <t>Gravier total extrait de la source : 72.06 T, reparti ici 1/3 (5/15) - 2/3 (5/25) a la demande de l'utilisateur (le fichier source ne distingue pas les 2 granulometries).</t>
+      </text>
+    </comment>
     <comment ref="C15" authorId="1" shapeId="0">
       <text>
         <t>Source : DALOT_2X3X2_L7.00_ml.xlsx, feuille 'MATERIAUX PRO' (ligne TOTAL) pour Ciment/Sable/Gravier, et 'RECAP FER' colonne BOTTES pour les aciers.</t>
+      </text>
+    </comment>
+    <comment ref="F15" authorId="2" shapeId="0">
+      <text>
+        <t>Gravier total extrait de la source : 105.79 T, reparti ici 1/3 (5/15) - 2/3 (5/25) a la demande de l'utilisateur (le fichier source ne distingue pas les 2 granulometries).</t>
       </text>
     </comment>
   </commentList>
@@ -634,16 +650,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:N22"/>
+  <dimension ref="B1:O22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
     <col width="8" customWidth="1" min="8" max="8"/>
     <col width="8" customWidth="1" min="9" max="9"/>
     <col width="8" customWidth="1" min="10" max="10"/>
@@ -651,6 +667,7 @@
     <col width="8" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="8" customWidth="1" min="14" max="14"/>
+    <col width="8" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -664,7 +681,7 @@
           <t>DS-MATERIAUX-GO</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>POLE OUVRAGE D'ART</t>
         </is>
@@ -688,14 +705,15 @@
       <c r="H3" s="5" t="n"/>
       <c r="I3" s="5" t="n"/>
       <c r="J3" s="5" t="n"/>
-      <c r="K3" s="4" t="inlineStr">
+      <c r="K3" s="5" t="n"/>
+      <c r="L3" s="4" t="inlineStr">
         <is>
           <t>N DS</t>
         </is>
       </c>
-      <c r="L3" s="5" t="n"/>
-      <c r="M3" s="6" t="n"/>
-      <c r="N3" s="5" t="n"/>
+      <c r="M3" s="5" t="n"/>
+      <c r="N3" s="6" t="n"/>
+      <c r="O3" s="5" t="n"/>
     </row>
     <row r="4">
       <c r="B4" s="4" t="inlineStr">
@@ -711,16 +729,17 @@
       <c r="H4" s="5" t="n"/>
       <c r="I4" s="5" t="n"/>
       <c r="J4" s="5" t="n"/>
-      <c r="K4" s="4" t="inlineStr">
+      <c r="K4" s="5" t="n"/>
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>Perte</t>
         </is>
       </c>
-      <c r="L4" s="5" t="n"/>
-      <c r="M4" s="9" t="n">
+      <c r="M4" s="5" t="n"/>
+      <c r="N4" s="9" t="n">
         <v>0.03</v>
       </c>
-      <c r="N4" s="5" t="n"/>
+      <c r="O4" s="5" t="n"/>
     </row>
     <row r="5" ht="14" customHeight="1">
       <c r="B5" s="10" t="inlineStr">
@@ -742,14 +761,15 @@
       <c r="H5" s="5" t="n"/>
       <c r="I5" s="5" t="n"/>
       <c r="J5" s="5" t="n"/>
-      <c r="K5" s="11" t="inlineStr">
+      <c r="K5" s="5" t="n"/>
+      <c r="L5" s="11" t="inlineStr">
         <is>
           <t>DALOT</t>
         </is>
       </c>
-      <c r="L5" s="5" t="n"/>
       <c r="M5" s="5" t="n"/>
       <c r="N5" s="5" t="n"/>
+      <c r="O5" s="5" t="n"/>
     </row>
     <row r="6" ht="14" customHeight="1">
       <c r="B6" s="5" t="n"/>
@@ -765,10 +785,11 @@
       <c r="H6" s="5" t="n"/>
       <c r="I6" s="5" t="n"/>
       <c r="J6" s="5" t="n"/>
-      <c r="K6" s="12" t="n"/>
-      <c r="L6" s="5" t="n"/>
+      <c r="K6" s="5" t="n"/>
+      <c r="L6" s="12" t="n"/>
       <c r="M6" s="5" t="n"/>
       <c r="N6" s="5" t="n"/>
+      <c r="O6" s="5" t="n"/>
     </row>
     <row r="7" ht="14" customHeight="1">
       <c r="B7" s="5" t="n"/>
@@ -784,10 +805,11 @@
       <c r="H7" s="5" t="n"/>
       <c r="I7" s="5" t="n"/>
       <c r="J7" s="5" t="n"/>
-      <c r="K7" s="12" t="n"/>
-      <c r="L7" s="5" t="n"/>
+      <c r="K7" s="5" t="n"/>
+      <c r="L7" s="12" t="n"/>
       <c r="M7" s="5" t="n"/>
       <c r="N7" s="5" t="n"/>
+      <c r="O7" s="5" t="n"/>
     </row>
     <row r="8" ht="14" customHeight="1">
       <c r="B8" s="5" t="n"/>
@@ -803,10 +825,11 @@
       <c r="H8" s="5" t="n"/>
       <c r="I8" s="5" t="n"/>
       <c r="J8" s="5" t="n"/>
-      <c r="K8" s="12" t="n"/>
-      <c r="L8" s="5" t="n"/>
+      <c r="K8" s="5" t="n"/>
+      <c r="L8" s="12" t="n"/>
       <c r="M8" s="5" t="n"/>
       <c r="N8" s="5" t="n"/>
+      <c r="O8" s="5" t="n"/>
     </row>
     <row r="10" ht="14" customHeight="1">
       <c r="B10" s="13" t="inlineStr">
@@ -834,73 +857,79 @@
           <t>GRAVIER</t>
         </is>
       </c>
-      <c r="G10" s="14" t="inlineStr">
+      <c r="G10" s="13" t="n"/>
+      <c r="H10" s="13" t="inlineStr">
         <is>
           <t>FER</t>
         </is>
       </c>
-      <c r="H10" s="14" t="n"/>
-      <c r="I10" s="14" t="n"/>
-      <c r="J10" s="14" t="n"/>
-      <c r="K10" s="14" t="n"/>
-      <c r="L10" s="14" t="n"/>
-      <c r="M10" s="14" t="n"/>
-      <c r="N10" s="14" t="n"/>
-    </row>
-    <row r="11" ht="14" customHeight="1">
+      <c r="I10" s="5" t="n"/>
+      <c r="J10" s="5" t="n"/>
+      <c r="K10" s="5" t="n"/>
+      <c r="L10" s="5" t="n"/>
+      <c r="M10" s="5" t="n"/>
+      <c r="N10" s="5" t="n"/>
+      <c r="O10" s="5" t="n"/>
+    </row>
+    <row r="11" ht="22" customHeight="1">
       <c r="B11" s="5" t="n"/>
       <c r="C11" s="5" t="n"/>
-      <c r="D11" s="15" t="inlineStr">
+      <c r="D11" s="14" t="inlineStr">
         <is>
           <t>en tonne</t>
         </is>
       </c>
-      <c r="E11" s="15" t="inlineStr">
+      <c r="E11" s="14" t="inlineStr">
         <is>
           <t>en tonne</t>
         </is>
       </c>
       <c r="F11" s="15" t="inlineStr">
         <is>
-          <t>en tonne</t>
-        </is>
-      </c>
-      <c r="G11" s="16" t="inlineStr">
+          <t>Gravier 5/15</t>
+        </is>
+      </c>
+      <c r="G11" s="15" t="inlineStr">
+        <is>
+          <t>Gravier 5/25</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
         <is>
           <t>HA 6</t>
         </is>
       </c>
-      <c r="H11" s="16" t="inlineStr">
+      <c r="I11" s="16" t="inlineStr">
         <is>
           <t>HA 8</t>
         </is>
       </c>
-      <c r="I11" s="16" t="inlineStr">
+      <c r="J11" s="16" t="inlineStr">
         <is>
           <t>HA 10</t>
         </is>
       </c>
-      <c r="J11" s="16" t="inlineStr">
+      <c r="K11" s="16" t="inlineStr">
         <is>
           <t>HA 12</t>
         </is>
       </c>
-      <c r="K11" s="16" t="inlineStr">
+      <c r="L11" s="16" t="inlineStr">
         <is>
           <t>HA 14</t>
         </is>
       </c>
-      <c r="L11" s="16" t="inlineStr">
+      <c r="M11" s="16" t="inlineStr">
         <is>
           <t>HA 16</t>
         </is>
       </c>
-      <c r="M11" s="16" t="inlineStr">
+      <c r="N11" s="16" t="inlineStr">
         <is>
           <t>HA 20</t>
         </is>
       </c>
-      <c r="N11" s="16" t="inlineStr">
+      <c r="O11" s="16" t="inlineStr">
         <is>
           <t>HA 25</t>
         </is>
@@ -911,8 +940,16 @@
       <c r="C12" s="5" t="n"/>
       <c r="D12" s="5" t="n"/>
       <c r="E12" s="5" t="n"/>
-      <c r="F12" s="5" t="n"/>
-      <c r="G12" s="5" t="n"/>
+      <c r="F12" s="14" t="inlineStr">
+        <is>
+          <t>en tonne</t>
+        </is>
+      </c>
+      <c r="G12" s="14" t="inlineStr">
+        <is>
+          <t>en tonne</t>
+        </is>
+      </c>
       <c r="H12" s="5" t="n"/>
       <c r="I12" s="5" t="n"/>
       <c r="J12" s="5" t="n"/>
@@ -920,6 +957,7 @@
       <c r="L12" s="5" t="n"/>
       <c r="M12" s="5" t="n"/>
       <c r="N12" s="5" t="n"/>
+      <c r="O12" s="5" t="n"/>
     </row>
     <row r="13" ht="26" customHeight="1">
       <c r="B13" s="7" t="inlineStr">
@@ -939,30 +977,33 @@
         <v>29.58</v>
       </c>
       <c r="F13" s="17" t="n">
-        <v>54.01</v>
+        <v>18</v>
       </c>
       <c r="G13" s="17" t="n">
+        <v>36.01</v>
+      </c>
+      <c r="H13" s="17" t="n">
         <v>0.2</v>
       </c>
-      <c r="H13" s="17" t="n">
+      <c r="I13" s="17" t="n">
         <v>1.7</v>
       </c>
-      <c r="I13" s="17" t="n">
+      <c r="J13" s="17" t="n">
         <v>10.8</v>
       </c>
-      <c r="J13" s="17" t="n">
+      <c r="K13" s="17" t="n">
         <v>19.9</v>
       </c>
-      <c r="K13" s="17" t="n">
+      <c r="L13" s="17" t="n">
         <v>3.8</v>
-      </c>
-      <c r="L13" s="17" t="n">
-        <v>0</v>
       </c>
       <c r="M13" s="17" t="n">
         <v>0</v>
       </c>
       <c r="N13" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="17" t="n">
         <v>0</v>
       </c>
     </row>
@@ -980,30 +1021,33 @@
         <v>39.35</v>
       </c>
       <c r="F14" s="17" t="n">
-        <v>72.06</v>
+        <v>24.02</v>
       </c>
       <c r="G14" s="17" t="n">
+        <v>48.04</v>
+      </c>
+      <c r="H14" s="17" t="n">
         <v>0.1</v>
       </c>
-      <c r="H14" s="17" t="n">
+      <c r="I14" s="17" t="n">
         <v>2.2</v>
       </c>
-      <c r="I14" s="17" t="n">
+      <c r="J14" s="17" t="n">
         <v>8.300000000000001</v>
       </c>
-      <c r="J14" s="17" t="n">
+      <c r="K14" s="17" t="n">
         <v>29.5</v>
       </c>
-      <c r="K14" s="17" t="n">
+      <c r="L14" s="17" t="n">
         <v>5.4</v>
       </c>
-      <c r="L14" s="17" t="n">
+      <c r="M14" s="17" t="n">
         <v>3.2</v>
       </c>
-      <c r="M14" s="17" t="n">
+      <c r="N14" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="N14" s="17" t="n">
+      <c r="O14" s="17" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1021,30 +1065,33 @@
         <v>53.23</v>
       </c>
       <c r="F15" s="17" t="n">
-        <v>105.79</v>
+        <v>35.26</v>
       </c>
       <c r="G15" s="17" t="n">
+        <v>70.52</v>
+      </c>
+      <c r="H15" s="17" t="n">
         <v>1.6</v>
       </c>
-      <c r="H15" s="17" t="n">
+      <c r="I15" s="17" t="n">
         <v>9.6</v>
       </c>
-      <c r="I15" s="17" t="n">
+      <c r="J15" s="17" t="n">
         <v>21.2</v>
       </c>
-      <c r="J15" s="17" t="n">
+      <c r="K15" s="17" t="n">
         <v>10.1</v>
       </c>
-      <c r="K15" s="17" t="n">
+      <c r="L15" s="17" t="n">
         <v>17.3</v>
       </c>
-      <c r="L15" s="17" t="n">
+      <c r="M15" s="17" t="n">
         <v>6.9</v>
       </c>
-      <c r="M15" s="17" t="n">
+      <c r="N15" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="N15" s="17" t="n">
+      <c r="O15" s="17" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1099,11 +1146,15 @@
         <f>SUM(N13:N15)</f>
         <v/>
       </c>
+      <c r="O16" s="22">
+        <f>SUM(O13:O15)</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="B18" s="23" t="inlineStr">
         <is>
-          <t>NOTE : le fichier source ne distingue pas les granulometries de gravillon (5/15 et 5/25) : la quantite de GRAVIER est donc regroupee dans une seule colonne (contrairement au modele d'origine qui separe Gravier 5/15 et Gravier 5/25). Les quantites d'aciers sont exprimees en 'Bottes' comme dans le modele fourni. Quantites nettes (hors perte).</t>
+          <t>NOTE : le fichier source ne distingue pas les granulometries de gravillon. La quantite totale de GRAVIER extraite a ete repartie ici 1/3 (Gravier 5/15) - 2/3 (Gravier 5/25) a la demande de l'utilisateur (voir commentaire sur chaque cellule 'Gravier 5/15' pour le total source). Les quantites d'aciers sont exprimees en 'Bottes' comme dans le modele fourni. Quantites nettes (hors perte).</t>
         </is>
       </c>
     </row>
@@ -1115,7 +1166,7 @@
           <t>IST</t>
         </is>
       </c>
-      <c r="K22" s="25" t="inlineStr">
+      <c r="L22" s="25" t="inlineStr">
         <is>
           <t>DIRECTION GENERALE</t>
         </is>
@@ -1123,46 +1174,46 @@
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="E1:J1"/>
+    <mergeCell ref="F5:K5"/>
     <mergeCell ref="B16:C16"/>
+    <mergeCell ref="L22:O22"/>
+    <mergeCell ref="F10:G10"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B1:D1"/>
     <mergeCell ref="M11:M12"/>
-    <mergeCell ref="K7:N7"/>
+    <mergeCell ref="L6:O6"/>
+    <mergeCell ref="H10:O10"/>
+    <mergeCell ref="F8:K8"/>
     <mergeCell ref="D11:D12"/>
-    <mergeCell ref="F6:J6"/>
-    <mergeCell ref="B22:F22"/>
+    <mergeCell ref="B19:O20"/>
     <mergeCell ref="H11:H12"/>
     <mergeCell ref="J11:J12"/>
-    <mergeCell ref="F7:J7"/>
-    <mergeCell ref="K6:N6"/>
+    <mergeCell ref="L3:M3"/>
+    <mergeCell ref="B18:O18"/>
+    <mergeCell ref="N3:O3"/>
     <mergeCell ref="K11:K12"/>
-    <mergeCell ref="F5:J5"/>
-    <mergeCell ref="G10:N10"/>
+    <mergeCell ref="L7:O7"/>
     <mergeCell ref="E11:E12"/>
-    <mergeCell ref="F8:J8"/>
-    <mergeCell ref="K5:N5"/>
-    <mergeCell ref="B19:N20"/>
-    <mergeCell ref="B18:N18"/>
+    <mergeCell ref="F3:K4"/>
+    <mergeCell ref="L4:M4"/>
+    <mergeCell ref="O11:O12"/>
     <mergeCell ref="D4:E4"/>
-    <mergeCell ref="M3:N3"/>
-    <mergeCell ref="K1:N1"/>
     <mergeCell ref="C10:C12"/>
-    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="E1:K1"/>
     <mergeCell ref="L11:L12"/>
     <mergeCell ref="B5:E8"/>
     <mergeCell ref="N11:N12"/>
-    <mergeCell ref="K22:N22"/>
-    <mergeCell ref="F3:J4"/>
+    <mergeCell ref="L5:O5"/>
+    <mergeCell ref="L8:O8"/>
+    <mergeCell ref="B22:G22"/>
+    <mergeCell ref="F6:K6"/>
     <mergeCell ref="B10:B12"/>
     <mergeCell ref="B13:B15"/>
-    <mergeCell ref="K8:N8"/>
-    <mergeCell ref="G11:G12"/>
-    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="F7:K7"/>
     <mergeCell ref="I11:I12"/>
-    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="L1:O1"/>
     <mergeCell ref="B4:C4"/>
-    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="N4:O4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>